<commit_message>
Update store rank list with ranks for all 93 stores
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016GtZZioynu6BNNHeRc885e
</commit_message>
<xml_diff>
--- a/store_rank_list.xlsx
+++ b/store_rank_list.xlsx
@@ -417,14 +417,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:D94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -448,94 +447,59 @@
           <t>エリア</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>シート</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>68</v>
+        <v>34</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>武庫川</t>
+          <t>宇部店</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>C</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>兵庫</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>関西</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>摂津南</t>
+          <t>浜田店</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>大阪</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>91</v>
+        <v>41</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>寝屋川</t>
+          <t>小月店</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>大阪</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>C</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>164</v>
+        <v>68</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>宝来</t>
+          <t>武庫川店</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -545,447 +509,312 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>奈良</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>兵庫</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>256</v>
+        <v>72</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>和泉</t>
+          <t>摂津南店</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
           <t>大阪</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>関西</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>270</v>
+        <v>74</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>半田亀崎</t>
+          <t>際波店</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>愛知</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>C</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>273</v>
+        <v>85</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>大和小泉</t>
+          <t>新下関店</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>奈良</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>299</v>
+        <v>90</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>四日市富田</t>
+          <t>東岡山店</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>三重</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>C</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>302</v>
+        <v>91</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>滋賀大津</t>
+          <t>寝屋川店</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>滋賀</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>大阪</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>308</v>
+        <v>123</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>松阪</t>
+          <t>防府店</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>三重</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>311</v>
+        <v>164</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>二色浜</t>
+          <t>宝来店</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>大阪</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>奈良</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>319</v>
+        <v>176</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>りんくう</t>
+          <t>琴浦店</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>大阪</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>C</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>324</v>
+        <v>227</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>安八</t>
+          <t>松江店</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
           <t>B</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>岐阜</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>中部</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>328</v>
+        <v>238</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>姫路</t>
+          <t>下松店</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>兵庫</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>333</v>
+        <v>256</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>東九条</t>
+          <t>和泉店</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>E</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>奈良</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>大阪</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>336</v>
+        <v>270</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>玉垣</t>
+          <t>半田亀崎店</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>三重</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>愛知</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>341</v>
+        <v>273</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>津藤方</t>
+          <t>大和小泉店</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>三重</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>奈良</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>367</v>
+        <v>298</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>彦根</t>
+          <t>鳥取千代水店</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
           <t>A</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>滋賀</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>関西</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>376</v>
+        <v>299</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>四日市南</t>
+          <t>四日市富田店</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
           <t>三重</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>中部</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>379</v>
+        <v>302</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>寝屋川大成</t>
+          <t>滋賀大津店</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>大阪</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>滋賀</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>386</v>
+        <v>306</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>久保</t>
+          <t>周南店</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>三重</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>B</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>387</v>
+        <v>308</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>阪南</t>
+          <t>松阪店</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -995,97 +824,72 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>大阪</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>三重</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>395</v>
+        <v>311</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>明石西インター</t>
+          <t>二色浜店</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>兵庫</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>大阪</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>406</v>
+        <v>319</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>湖南</t>
+          <t>りんくうタウン店</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>滋賀</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>大阪</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>410</v>
+        <v>321</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>近江八幡</t>
+          <t>米子大谷店</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
           <t>B</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>滋賀</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>関西</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>417</v>
+        <v>324</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>幸田</t>
+          <t>安八店</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1095,72 +899,52 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>愛知</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>岐阜</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>422</v>
+        <v>328</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>養父</t>
+          <t>姫路店</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
           <t>兵庫</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>中四国</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>423</v>
+        <v>329</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>岐南八剣</t>
+          <t>大竹店</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>岐阜</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>437</v>
+        <v>333</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>伊勢</t>
+          <t>東九条店</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1170,47 +954,32 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>三重</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>奈良</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>454</v>
+        <v>334</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>三田</t>
+          <t>出雲斐川店</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
           <t>B</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>兵庫</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>関西</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>456</v>
+        <v>336</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>箕面森町</t>
+          <t>玉垣店</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1220,22 +989,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>大阪</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>三重</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>462</v>
+        <v>341</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>橿原</t>
+          <t>津藤方店</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1245,122 +1009,82 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>奈良</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>三重</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>466</v>
+        <v>349</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>桜井粟殿</t>
+          <t>境港店</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
           <t>C</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>奈良</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>関西</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>467</v>
+        <v>357</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>御所</t>
+          <t>宇部中央店</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>奈良</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>C</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>469</v>
+        <v>367</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>関</t>
+          <t>彦根店</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>岐阜</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>滋賀</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>478</v>
+        <v>375</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>みえ朝日</t>
+          <t>出雲白枝店</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>三重</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>480</v>
+        <v>376</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>天理</t>
+          <t>四日市南店</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1370,47 +1094,32 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>奈良</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>三重</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>481</v>
+        <v>377</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>富田林</t>
+          <t>東岐波店</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
           <t>A</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>大阪</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>関西</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>497</v>
+        <v>379</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>オーキッドパーク</t>
+          <t>寝屋川大成店</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1420,47 +1129,37 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>岐阜</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>大阪</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>529</v>
+        <v>386</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>名古屋茶屋</t>
+          <t>久保店</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>岐阜</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>三重</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>547</v>
+        <v>387</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>草津矢橋</t>
+          <t>阪南店</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1470,47 +1169,32 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>滋賀</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>大阪</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>555</v>
+        <v>390</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>赤穂</t>
+          <t>叶店</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
           <t>C</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>滋賀</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>関西</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>579</v>
+        <v>395</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>岩出</t>
+          <t>明石西インター店</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1520,237 +1204,902 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>和歌山</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>兵庫</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>667</v>
+        <v>401</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>丸亀</t>
+          <t>益田店</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
           <t>C</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>香川</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>中四国</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>690</v>
+        <v>406</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>大府</t>
+          <t>湖南店</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>愛知</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>滋賀</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>697</v>
+        <v>410</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>富山マイプラザ</t>
+          <t>近江八幡店</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>富山</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>滋賀</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>707</v>
+        <v>411</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>野々市</t>
+          <t>柳井店</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>石川</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>関西</t>
+          <t>A</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>713</v>
+        <v>417</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>善通寺</t>
+          <t>幸田店</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>香川</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>中四国</t>
+          <t>愛知</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>727</v>
+        <v>422</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>浜松若林</t>
+          <t>養父店</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>静岡</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>兵庫</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>745</v>
+        <v>423</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>三豊</t>
+          <t>岐南八剣店</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>香川</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>中四国</t>
+          <t>岐阜</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>755</v>
+        <v>437</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>掛川</t>
+          <t>伊勢店</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>C</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>静岡</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>中部</t>
+          <t>三重</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
+        <v>440</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>雲南店</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>454</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>三田店</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>兵庫</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>456</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>箕面森町店</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>大阪</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>462</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>橿原店</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>奈良</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>466</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>桜井粟殿店</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>奈良</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>467</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>御所店</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>奈良</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>469</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>関店</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>岐阜</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>474</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>長府店</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>478</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>みえ朝日店</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>三重</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>480</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>天理店</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>奈良</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>481</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>富田林店</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>大阪</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>497</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>オーキッドパーク店</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>岐阜</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>529</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>名古屋茶屋店</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>岐阜</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>547</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>草津矢橋店</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>滋賀</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>555</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>赤穂店</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>滋賀</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>558</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>鳥取大杙店</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>579</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>岩出店</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>和歌山</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>667</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>丸亀店</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>香川</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>677</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>下関生野店</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>690</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>大府店</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>愛知</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>697</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>富山マイプラザ店</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>富山</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>707</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>野々市店</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>石川</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>713</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>善通寺店</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>香川</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>716</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>守口ジャガータウン店</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>727</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>浜松若林店</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>静岡</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>745</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>三豊店</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>香川</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>751</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>大田店</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>755</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>掛川店</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>静岡</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
         <v>758</v>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>三木</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>三木店</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
         <is>
           <t>香川</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>中四国</t>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>763</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>岡山豊浜店</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>770</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>平群店</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>771</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>西条店</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>772</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>西尾一色店</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>774</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>板野店</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>775</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>西大和店</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>802</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>浜北店</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>806</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>姫路四郷店</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>812</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>阿波土成店</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>813</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>浜松葵西店</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>815</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>本巣店</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>816</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>松山空港通り店</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>817</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>名張店</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>A</t>
         </is>
       </c>
     </row>

</xml_diff>